<commit_message>
Fix MN-2007 bridge: use CCSS + anchor-level MN-2022 mapping
- Bridge now uses CCSS-M codes AND MN-2022 anchor standards (not whole strands)
- CC1 2.3.2-2.3.4 now correctly show MN-2007 alignments
- CC1 1.2.1-1.2.3 now show Fractions via CCSS bridge
- Max standards per module: 6 (was 14+ with old broad bridge)
- MN-2007 Grade 6: 18/18, Grade 7: 15/18, Grade 8: 14/16
- 945 MN-2007 alignments via targeted bridge

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/viewer/downloads/CC1_Alignment.xlsx
+++ b/viewer/downloads/CC1_Alignment.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation_supplement</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation_supplement</t>
         </is>
       </c>
     </row>
@@ -742,12 +742,12 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>6.NS.B.4 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -769,12 +769,12 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>6.NS.B.4 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -800,12 +800,12 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>6.NS.B.4 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -835,12 +835,12 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.4 (MN-2022), 6.EE.A.1 (CCSS-M), 6.EE.A.2.B (CCSS-M), 6.NS.B.4 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.4 (MN-2022), 6.EE.A.1 (CCSS-M), 6.EE.A.2.B (CCSS-M), 6.NS.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -883,12 +883,12 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.4 (MN-2022), 6.2.3.5 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.SP.B.4 (CCSS-M)</t>
+          <t>6.1.1.4 (MN-2022), 6.2.3.5 (MN-2022), 6.3.2.1 (MN-2007), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.SP.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation, mn_correlation_supplement</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation, mn_correlation_supplement</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation_supplement</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation_supplement</t>
         </is>
       </c>
     </row>
@@ -949,12 +949,12 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>6.G.A.1 (CCSS-M)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -984,12 +984,12 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.1 (MN-2022), 6.G.A.1 (CCSS-M)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.6.1 (MN-2022), 6.G.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.5 (MN-2022), 6.G.A.1 (CCSS-M)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.5.5 (MN-2022), 6.G.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1050,12 +1050,12 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>6.EE.A.3 (CCSS-M), 6.NS.B.2 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.3 (CCSS-M), 6.NS.B.2 (CCSS-M)</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1081,12 +1081,12 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>6.EE.A.3 (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.3 (CCSS-M)</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1112,12 +1112,12 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>6.NS.B.4 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1143,12 +1143,12 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>6.EE.A.3 (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.3 (CCSS-M)</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1191,12 +1191,12 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.5 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
+          <t>6.1.1.4 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.5 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
+          <t>6.1.1.4 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1261,12 +1261,12 @@
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.2 (MN-2022), 6.NS.B.3 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.2 (MN-2022), 6.NS.B.3 (CCSS-M)</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1292,12 +1292,12 @@
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>6.NS.B.3 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.B.3 (CCSS-M)</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1327,12 @@
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.2 (MN-2022), 6.NS.B.3 (CCSS-M), 6.RP.A.3.C (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.3 (MN-2007), 6.3.6.2 (MN-2022), 6.NS.B.3 (CCSS-M), 6.RP.A.3.C (CCSS-M)</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.2 (MN-2022), 6.3.6.5 (MN-2022), 6.RP.A.1 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.2 (MN-2022), 6.3.6.5 (MN-2022), 6.RP.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1397,12 +1397,12 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.1 (MN-2022), 6.3.5.2 (MN-2022), 6.NS.C.6.A (CCSS-M), 6.NS.C.6.B (CCSS-M)</t>
+          <t>6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.1 (MN-2022), 6.3.5.2 (MN-2022), 6.NS.C.6.A (CCSS-M), 6.NS.C.6.B (CCSS-M)</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1432,12 @@
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.5 (MN-2022), 6.NS.C.5 (CCSS-M), 6.NS.C.6.A (CCSS-M), 6.NS.C.7.A (CCSS-M)</t>
+          <t>6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.5 (MN-2022), 6.NS.C.5 (CCSS-M), 6.NS.C.6.A (CCSS-M), 6.NS.C.7.A (CCSS-M)</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1467,12 +1467,12 @@
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.NS.C.7.B (CCSS-M), 6.NS.C.7.C (CCSS-M), 6.NS.C.7.D (CCSS-M)</t>
+          <t>6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.NS.C.7.B (CCSS-M), 6.NS.C.7.C (CCSS-M), 6.NS.C.7.D (CCSS-M)</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1502,12 +1502,12 @@
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.2.4.3 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.1 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.6 (MN-2022), 6.NS.C.6.B (CCSS-M), 6.NS.C.6.C (CCSS-M), 6.NS.C.8 (CCSS-M)</t>
+          <t>6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.4.3 (MN-2022), 6.3.2.1 (MN-2007), 6.3.5.1 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.6 (MN-2022), 6.NS.C.6.B (CCSS-M), 6.NS.C.6.C (CCSS-M), 6.NS.C.8 (CCSS-M)</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1550,12 +1550,12 @@
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.2 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.EE.A.2.A (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
+          <t>6.1.2.2 (MN-2022), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.2.A (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1581,12 +1581,12 @@
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>6.EE.A.4 (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.4 (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
         </is>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1616,12 +1616,12 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.1 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.EE.A.2.A (CCSS-M), 6.EE.A.2.C (CCSS-M), 6.EE.A.4 (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2022), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.2.A (CCSS-M), 6.EE.A.2.C (CCSS-M), 6.EE.A.4 (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1647,12 +1647,12 @@
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>6.RP.A.1 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.RP.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1678,12 +1678,12 @@
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>6.RP.A.1 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.RP.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1709,12 +1709,12 @@
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>6.RP.A.1 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.RP.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1740,12 +1740,12 @@
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>6.RP.A.1 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.RP.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1788,12 +1788,12 @@
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
+          <t>6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1842,12 +1842,12 @@
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
+          <t>6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1908,12 +1908,12 @@
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.5 (MN-2022), 6.NS.3 (CCSS-M), 6.RP.3c (CCSS-M)</t>
+          <t>6.3.6.5 (MN-2022), 6.NS.3 (CCSS-M), 6.RP.3c (CCSS-M)</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
+          <t>ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2164,12 +2164,12 @@
       <c r="E58" s="8" t="inlineStr"/>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.7 (MN-2022)</t>
+          <t>6.3.5.7 (MN-2022)</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2195,12 +2195,12 @@
       <c r="E59" s="8" t="inlineStr"/>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022)</t>
+          <t>6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2298,7 @@
       <c r="E64" s="8" t="inlineStr"/>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.5 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007)</t>
+          <t>6.2.3.5 (MN-2022), 6.3.2.1 (MN-2007)</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
@@ -2342,12 +2342,12 @@
       <c r="E66" s="8" t="inlineStr"/>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.1 (MN-2022), 6.1.2.2 (MN-2007), 6.1.2.2 (MN-2022), 6.1.2.3 (MN-2007), 6.1.2.3 (MN-2022), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.11 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+          <t>6.1.2.1 (MN-2022), 6.1.2.2 (MN-2022), 6.1.2.3 (MN-2022), 6.3.5.11 (MN-2022)</t>
         </is>
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2407,12 +2407,12 @@
       <c r="E69" s="8" t="inlineStr"/>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.3 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+          <t>6.1.2.3 (MN-2022)</t>
         </is>
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2587,7 +2587,7 @@
       <c r="E79" s="8" t="inlineStr"/>
       <c r="F79" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.3 (MN-2022), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.9 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+          <t>6.1.1.3 (MN-2022), 6.3.5.9 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
         </is>
       </c>
       <c r="G79" s="8" t="inlineStr">
@@ -2618,7 +2618,7 @@
       <c r="E80" s="8" t="inlineStr"/>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.1.5 (MN-2022), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+          <t>6.1.1.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
         </is>
       </c>
       <c r="G80" s="8" t="inlineStr">
@@ -2668,7 +2668,7 @@
       <c r="E82" s="8" t="inlineStr"/>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.3 (MN-2022), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.2.3.4 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.8 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+          <t>6.1.1.3 (MN-2022), 6.2.3.4 (MN-2022), 6.3.2.1 (MN-2007), 6.3.5.8 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
         </is>
       </c>
       <c r="G82" s="8" t="inlineStr">
@@ -2730,7 +2730,7 @@
       <c r="E84" s="8" t="inlineStr"/>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.1 (MN-2022), 6.1.1.2 (MN-2007), 6.1.1.2 (MN-2022), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2022), 6.1.1.2 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
         </is>
       </c>
       <c r="G84" s="8" t="inlineStr">
@@ -2819,7 +2819,7 @@
       <c r="E89" s="8" t="inlineStr"/>
       <c r="F89" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.2.3.4 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.9 (MN-2022)</t>
+          <t>6.2.3.4 (MN-2022), 6.3.2.1 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.9 (MN-2022)</t>
         </is>
       </c>
       <c r="G89" s="8" t="inlineStr">
@@ -2850,12 +2850,12 @@
       <c r="E90" s="8" t="inlineStr"/>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.9 (MN-2022)</t>
+          <t>6.3.5.9 (MN-2022)</t>
         </is>
       </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2881,12 +2881,12 @@
       <c r="E91" s="8" t="inlineStr"/>
       <c r="F91" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022)</t>
+          <t>6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022)</t>
         </is>
       </c>
       <c r="G91" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       <c r="E92" s="8" t="inlineStr"/>
       <c r="F92" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.2.3.4 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.7 (MN-2022)</t>
+          <t>6.2.3.4 (MN-2022), 6.3.2.1 (MN-2007), 6.3.5.7 (MN-2022)</t>
         </is>
       </c>
       <c r="G92" s="8" t="inlineStr">
@@ -2962,12 +2962,12 @@
       <c r="E94" s="8" t="inlineStr"/>
       <c r="F94" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022)</t>
+          <t>6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022)</t>
         </is>
       </c>
       <c r="G94" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2989,12 +2989,12 @@
       <c r="E95" s="8" t="inlineStr"/>
       <c r="F95" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022)</t>
+          <t>6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -3016,12 +3016,12 @@
       <c r="E96" s="8" t="inlineStr"/>
       <c r="F96" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.1 (MN-2022), 6.3.7.1 (MN-2022)</t>
+          <t>6.3.6.1 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -3043,12 +3043,12 @@
       <c r="E97" s="8" t="inlineStr"/>
       <c r="F97" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.1 (MN-2022)</t>
+          <t>6.3.6.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       <c r="E99" s="8" t="inlineStr"/>
       <c r="F99" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.2.3.3 (MN-2022), 6.2.3.4 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.10 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022)</t>
+          <t>6.2.3.3 (MN-2022), 6.2.3.4 (MN-2022), 6.3.2.1 (MN-2007), 6.3.5.10 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G99" s="8" t="inlineStr">
@@ -3110,12 +3110,12 @@
       <c r="E100" s="8" t="inlineStr"/>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>6.2.4.1 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007)</t>
+          <t>6.2.4.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -3137,12 +3137,12 @@
       <c r="E101" s="8" t="inlineStr"/>
       <c r="F101" s="8" t="inlineStr">
         <is>
-          <t>6.2.4.2 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007)</t>
+          <t>6.2.4.2 (MN-2022)</t>
         </is>
       </c>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
       <c r="E103" s="8" t="inlineStr"/>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007)</t>
+          <t>6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022), 6.3.2.1 (MN-2007)</t>
         </is>
       </c>
       <c r="G103" s="8" t="inlineStr">
@@ -3204,12 +3204,12 @@
       <c r="E104" s="8" t="inlineStr"/>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022)</t>
+          <t>6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_mn2022, mn_correlation</t>
+          <t>mn_correlation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix MN-2007 bridge: CCSS code normalization, HS ID collision, domain-based MN-2022 mapping
Three bugs fixed in the MN-2007 alignment bridge:
- CCSS short-form codes (6.G.1) now match full-form (6.G.A.1) in cross-reference
- HS MN-2007 standard IDs no longer collide with CCSS entries
- MN-2022 numeric→strand-letter mapping replaced with domain-based cluster matching

Added content-based bridge for 26 lessons missing all source alignment data.
Added correlation strength indicators (STRONG/MEDIUM/INFERRED) to viewer tags.

MN-2007 coverage: CC1 58→90%, CCA/CCG/CCA2 0→79-93%.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/viewer/downloads/CC1_Alignment.xlsx
+++ b/viewer/downloads/CC1_Alignment.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.4 (MN-2022), 6.2.3.5 (MN-2022), 6.3.2.1 (MN-2007), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.SP.B.4 (CCSS-M)</t>
+          <t>6.1.1.4 (MN-2022), 6.2.3.5 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.SP.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
@@ -984,12 +984,12 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.6.1 (MN-2022), 6.G.A.1 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.6.1 (MN-2022), 6.G.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.5.5 (MN-2022), 6.G.A.1 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.5.5 (MN-2022), 6.G.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1191,12 +1191,12 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.4 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.5 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.5 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.4 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022), 6.RP.A.3.C (CCSS-M)</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
@@ -1261,12 +1261,12 @@
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.2 (MN-2022), 6.NS.B.3 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.2 (MN-2022), 6.NS.B.3 (CCSS-M)</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.3 (MN-2007), 6.3.6.2 (MN-2022), 6.NS.B.3 (CCSS-M), 6.RP.A.3.C (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.6.2 (MN-2022), 6.NS.B.3 (CCSS-M), 6.RP.A.3.C (CCSS-M)</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -1397,12 +1397,12 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.1 (MN-2022), 6.3.5.2 (MN-2022), 6.NS.C.6.A (CCSS-M), 6.NS.C.6.B (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.1 (MN-2022), 6.3.5.2 (MN-2022), 6.NS.C.6.A (CCSS-M), 6.NS.C.6.B (CCSS-M)</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1432,12 @@
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.5 (MN-2022), 6.NS.C.5 (CCSS-M), 6.NS.C.6.A (CCSS-M), 6.NS.C.7.A (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.5 (MN-2022), 6.NS.C.5 (CCSS-M), 6.NS.C.6.A (CCSS-M), 6.NS.C.7.A (CCSS-M)</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1467,12 +1467,12 @@
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.NS.C.7.B (CCSS-M), 6.NS.C.7.C (CCSS-M), 6.NS.C.7.D (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.NS.C.7.B (CCSS-M), 6.NS.C.7.C (CCSS-M), 6.NS.C.7.D (CCSS-M)</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1502,12 +1502,12 @@
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.4.3 (MN-2022), 6.3.2.1 (MN-2007), 6.3.5.1 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.6 (MN-2022), 6.NS.C.6.B (CCSS-M), 6.NS.C.6.C (CCSS-M), 6.NS.C.8 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.1.3.1 (MN-2007), 6.1.3.2 (MN-2007), 6.1.3.3 (MN-2007), 6.2.4.3 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.1 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.6 (MN-2022), 6.NS.C.6.B (CCSS-M), 6.NS.C.6.C (CCSS-M), 6.NS.C.8 (CCSS-M)</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1550,12 +1550,12 @@
       </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.2 (MN-2022), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.2.A (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
+          <t>6.1.2.2 (MN-2022), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.EE.A.2.A (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1616,12 +1616,12 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.1 (MN-2022), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.2.A (CCSS-M), 6.EE.A.2.C (CCSS-M), 6.EE.A.4 (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2022), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007), 6.EE.A.2.A (CCSS-M), 6.EE.A.2.C (CCSS-M), 6.EE.A.4 (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>bridged_via_ccss, ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1788,12 +1788,12 @@
       </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1813,8 +1813,16 @@
       </c>
       <c r="D45" s="8" t="inlineStr"/>
       <c r="E45" s="8" t="inlineStr"/>
-      <c r="F45" s="8" t="inlineStr"/>
-      <c r="G45" s="8" t="inlineStr"/>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -1842,12 +1850,12 @@
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1873,12 +1881,12 @@
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>Review skills needed for 6.NS.1 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), Review skills needed for 6.NS.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1908,12 +1916,12 @@
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.5 (MN-2022), 6.NS.3 (CCSS-M), 6.RP.3c (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.6.5 (MN-2022), 6.NS.3 (CCSS-M), 6.RP.3c (CCSS-M)</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide, mn_correlation</t>
+          <t>bridged_via_ccss, bridged_via_mn2022, ccss_lesson_guide, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -1939,12 +1947,12 @@
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>Review skills needed for 6.NS.1 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), Review skills needed for 6.NS.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -1970,12 +1978,12 @@
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>6.G.1 (CCSS-M)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -2001,12 +2009,12 @@
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>6.G.1 (CCSS-M)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -2032,12 +2040,12 @@
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>6.G.1 (CCSS-M)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -2063,12 +2071,12 @@
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>6.G.1 (CCSS-M)</t>
+          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>ccss_lesson_guide</t>
+          <t>bridged_via_ccss, ccss_lesson_guide</t>
         </is>
       </c>
     </row>
@@ -2101,8 +2109,16 @@
       </c>
       <c r="D55" s="8" t="inlineStr"/>
       <c r="E55" s="8" t="inlineStr"/>
-      <c r="F55" s="8" t="inlineStr"/>
-      <c r="G55" s="8" t="inlineStr"/>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">
@@ -2120,8 +2136,16 @@
       </c>
       <c r="D56" s="8" t="inlineStr"/>
       <c r="E56" s="8" t="inlineStr"/>
-      <c r="F56" s="8" t="inlineStr"/>
-      <c r="G56" s="8" t="inlineStr"/>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G56" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -2139,8 +2163,16 @@
       </c>
       <c r="D57" s="8" t="inlineStr"/>
       <c r="E57" s="8" t="inlineStr"/>
-      <c r="F57" s="8" t="inlineStr"/>
-      <c r="G57" s="8" t="inlineStr"/>
+      <c r="F57" s="8" t="inlineStr">
+        <is>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G57" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n">
@@ -2164,12 +2196,12 @@
       <c r="E58" s="8" t="inlineStr"/>
       <c r="F58" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.7 (MN-2022)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.7 (MN-2022)</t>
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2195,12 +2227,12 @@
       <c r="E59" s="8" t="inlineStr"/>
       <c r="F59" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2220,8 +2252,16 @@
       </c>
       <c r="D60" s="8" t="inlineStr"/>
       <c r="E60" s="8" t="inlineStr"/>
-      <c r="F60" s="8" t="inlineStr"/>
-      <c r="G60" s="8" t="inlineStr"/>
+      <c r="F60" s="8" t="inlineStr">
+        <is>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G60" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n">
@@ -2239,8 +2279,16 @@
       </c>
       <c r="D61" s="8" t="inlineStr"/>
       <c r="E61" s="8" t="inlineStr"/>
-      <c r="F61" s="8" t="inlineStr"/>
-      <c r="G61" s="8" t="inlineStr"/>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G61" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n">
@@ -2258,8 +2306,16 @@
       </c>
       <c r="D62" s="8" t="inlineStr"/>
       <c r="E62" s="8" t="inlineStr"/>
-      <c r="F62" s="8" t="inlineStr"/>
-      <c r="G62" s="8" t="inlineStr"/>
+      <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G62" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n">
@@ -2277,8 +2333,16 @@
       </c>
       <c r="D63" s="8" t="inlineStr"/>
       <c r="E63" s="8" t="inlineStr"/>
-      <c r="F63" s="8" t="inlineStr"/>
-      <c r="G63" s="8" t="inlineStr"/>
+      <c r="F63" s="8" t="inlineStr">
+        <is>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G63" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n">
@@ -2298,7 +2362,7 @@
       <c r="E64" s="8" t="inlineStr"/>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.5 (MN-2022), 6.3.2.1 (MN-2007)</t>
+          <t>6.2.3.5 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007)</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
@@ -2342,12 +2406,12 @@
       <c r="E66" s="8" t="inlineStr"/>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.1 (MN-2022), 6.1.2.2 (MN-2022), 6.1.2.3 (MN-2022), 6.3.5.11 (MN-2022)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.1 (MN-2022), 6.1.2.2 (MN-2007), 6.1.2.2 (MN-2022), 6.1.2.3 (MN-2007), 6.1.2.3 (MN-2022), 6.3.5.11 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
         </is>
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2367,8 +2431,16 @@
       </c>
       <c r="D67" s="8" t="inlineStr"/>
       <c r="E67" s="8" t="inlineStr"/>
-      <c r="F67" s="8" t="inlineStr"/>
-      <c r="G67" s="8" t="inlineStr"/>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G67" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="n">
@@ -2386,8 +2458,16 @@
       </c>
       <c r="D68" s="8" t="inlineStr"/>
       <c r="E68" s="8" t="inlineStr"/>
-      <c r="F68" s="8" t="inlineStr"/>
-      <c r="G68" s="8" t="inlineStr"/>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G68" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n">
@@ -2407,12 +2487,12 @@
       <c r="E69" s="8" t="inlineStr"/>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.3 (MN-2022)</t>
+          <t>6.1.2.3 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
         </is>
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2432,8 +2512,16 @@
       </c>
       <c r="D70" s="8" t="inlineStr"/>
       <c r="E70" s="8" t="inlineStr"/>
-      <c r="F70" s="8" t="inlineStr"/>
-      <c r="G70" s="8" t="inlineStr"/>
+      <c r="F70" s="8" t="inlineStr">
+        <is>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G70" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n">
@@ -2451,8 +2539,16 @@
       </c>
       <c r="D71" s="8" t="inlineStr"/>
       <c r="E71" s="8" t="inlineStr"/>
-      <c r="F71" s="8" t="inlineStr"/>
-      <c r="G71" s="8" t="inlineStr"/>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G71" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n">
@@ -2470,8 +2566,16 @@
       </c>
       <c r="D72" s="8" t="inlineStr"/>
       <c r="E72" s="8" t="inlineStr"/>
-      <c r="F72" s="8" t="inlineStr"/>
-      <c r="G72" s="8" t="inlineStr"/>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G72" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n">
@@ -2489,8 +2593,16 @@
       </c>
       <c r="D73" s="8" t="inlineStr"/>
       <c r="E73" s="8" t="inlineStr"/>
-      <c r="F73" s="8" t="inlineStr"/>
-      <c r="G73" s="8" t="inlineStr"/>
+      <c r="F73" s="8" t="inlineStr">
+        <is>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G73" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n">
@@ -2587,7 +2699,7 @@
       <c r="E79" s="8" t="inlineStr"/>
       <c r="F79" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.3 (MN-2022), 6.3.5.9 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.3 (MN-2022), 6.3.5.9 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
         </is>
       </c>
       <c r="G79" s="8" t="inlineStr">
@@ -2618,7 +2730,7 @@
       <c r="E80" s="8" t="inlineStr"/>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
         </is>
       </c>
       <c r="G80" s="8" t="inlineStr">
@@ -2643,8 +2755,16 @@
       </c>
       <c r="D81" s="8" t="inlineStr"/>
       <c r="E81" s="8" t="inlineStr"/>
-      <c r="F81" s="8" t="inlineStr"/>
-      <c r="G81" s="8" t="inlineStr"/>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G81" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n">
@@ -2668,7 +2788,7 @@
       <c r="E82" s="8" t="inlineStr"/>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.3 (MN-2022), 6.2.3.4 (MN-2022), 6.3.2.1 (MN-2007), 6.3.5.8 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.3 (MN-2022), 6.2.3.4 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.8 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
         </is>
       </c>
       <c r="G82" s="8" t="inlineStr">
@@ -2730,7 +2850,7 @@
       <c r="E84" s="8" t="inlineStr"/>
       <c r="F84" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2022), 6.1.1.2 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.1 (MN-2022), 6.1.1.2 (MN-2007), 6.1.1.2 (MN-2022), 6.1.1.3 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.4.1.1 (MN-2007), 6.4.1.2 (MN-2007)</t>
         </is>
       </c>
       <c r="G84" s="8" t="inlineStr">
@@ -2819,7 +2939,7 @@
       <c r="E89" s="8" t="inlineStr"/>
       <c r="F89" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.4 (MN-2022), 6.3.2.1 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.9 (MN-2022)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.2.3.4 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.9 (MN-2022)</t>
         </is>
       </c>
       <c r="G89" s="8" t="inlineStr">
@@ -2850,12 +2970,12 @@
       <c r="E90" s="8" t="inlineStr"/>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.9 (MN-2022)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.9 (MN-2022)</t>
         </is>
       </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2881,12 +3001,12 @@
       <c r="E91" s="8" t="inlineStr"/>
       <c r="F91" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022)</t>
         </is>
       </c>
       <c r="G91" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2912,7 +3032,7 @@
       <c r="E92" s="8" t="inlineStr"/>
       <c r="F92" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.4 (MN-2022), 6.3.2.1 (MN-2007), 6.3.5.7 (MN-2022)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.2.3.4 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.7 (MN-2022)</t>
         </is>
       </c>
       <c r="G92" s="8" t="inlineStr">
@@ -2937,8 +3057,16 @@
       </c>
       <c r="D93" s="8" t="inlineStr"/>
       <c r="E93" s="8" t="inlineStr"/>
-      <c r="F93" s="8" t="inlineStr"/>
-      <c r="G93" s="8" t="inlineStr"/>
+      <c r="F93" s="8" t="inlineStr">
+        <is>
+          <t>6.1.1.4 (MN-2007)</t>
+        </is>
+      </c>
+      <c r="G93" s="8" t="inlineStr">
+        <is>
+          <t>bridged_via_content</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="n">
@@ -2962,12 +3090,12 @@
       <c r="E94" s="8" t="inlineStr"/>
       <c r="F94" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022)</t>
         </is>
       </c>
       <c r="G94" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -2989,12 +3117,12 @@
       <c r="E95" s="8" t="inlineStr"/>
       <c r="F95" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -3016,12 +3144,12 @@
       <c r="E96" s="8" t="inlineStr"/>
       <c r="F96" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.1 (MN-2022), 6.3.7.1 (MN-2022)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.6.1 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -3043,12 +3171,12 @@
       <c r="E97" s="8" t="inlineStr"/>
       <c r="F97" s="8" t="inlineStr">
         <is>
-          <t>6.3.6.1 (MN-2022)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.6.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3211,7 @@
       <c r="E99" s="8" t="inlineStr"/>
       <c r="F99" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.3 (MN-2022), 6.2.3.4 (MN-2022), 6.3.2.1 (MN-2007), 6.3.5.10 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.2.3.3 (MN-2022), 6.2.3.4 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007), 6.3.5.10 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G99" s="8" t="inlineStr">
@@ -3110,12 +3238,12 @@
       <c r="E100" s="8" t="inlineStr"/>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>6.2.4.1 (MN-2022)</t>
+          <t>6.2.4.1 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007)</t>
         </is>
       </c>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -3137,12 +3265,12 @@
       <c r="E101" s="8" t="inlineStr"/>
       <c r="F101" s="8" t="inlineStr">
         <is>
-          <t>6.2.4.2 (MN-2022)</t>
+          <t>6.2.4.2 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007)</t>
         </is>
       </c>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3305,7 @@
       <c r="E103" s="8" t="inlineStr"/>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022), 6.3.2.1 (MN-2007)</t>
+          <t>6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.3.2.1 (MN-2007)</t>
         </is>
       </c>
       <c r="G103" s="8" t="inlineStr">
@@ -3204,12 +3332,12 @@
       <c r="E104" s="8" t="inlineStr"/>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>mn_correlation</t>
+          <t>bridged_via_mn2022, mn_correlation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add CCSS→MN-2022 bridge, fill alignment gaps across all frameworks
- CCSS→MN-2022 bridge: 913 new alignments using cross-reference map
  with description-based narrowing (not whole-domain dumps)
- Content→MN-2022 bridge: 250 alignments for lessons with no source data
- Embedded heatmap into By Grade and By Book views (red→green gradient)
- Removed standalone heatmap tab and strength badges
- Fixed: lessons like 2.2.1 "Area of Polygons" now properly aligned

MN-2022 coverage: CC1 72%→89%, CC2 47%→90%, CC3 55%→96%

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/viewer/downloads/CC1_Alignment.xlsx
+++ b/viewer/downloads/CC1_Alignment.xlsx
@@ -734,7 +734,11 @@
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr"/>
-      <c r="D10" s="8" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
           <t>6.NS.B.4</t>
@@ -742,7 +746,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.B.4 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022), 6.NS.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -761,7 +765,11 @@
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr"/>
-      <c r="D11" s="8" t="inlineStr"/>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
           <t>6.NS.B.4</t>
@@ -769,7 +777,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.B.4 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022), 6.NS.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -792,7 +800,11 @@
           <t>Number Sense</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr"/>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
           <t>6.NS.B.4</t>
@@ -800,7 +812,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.B.4 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022), 6.NS.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -941,7 +953,11 @@
           <t>Area of Polygons</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>6.2.3.1, 6.2.3.2, 6.2.3.3, 6.2.3.4, 6.2.3.5, 6.2.4.1, 6.2.4.2, 6.2.4.3</t>
+        </is>
+      </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
           <t>6.G.A.1</t>
@@ -949,7 +965,7 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.A.1 (CCSS-M)</t>
+          <t>6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022), 6.2.3.3 (MN-2022), 6.2.3.4 (MN-2022), 6.2.3.5 (MN-2022), 6.2.4.1 (MN-2022), 6.2.4.2 (MN-2022), 6.2.4.3 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -1042,7 +1058,11 @@
           <t>Multiplying Multi-Digit Numbers</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.3, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.6, 6.3.7.1</t>
+        </is>
+      </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
           <t>6.EE.A.3, 6.NS.B.2</t>
@@ -1050,7 +1070,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.3 (CCSS-M), 6.NS.B.2 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.6 (MN-2022), 6.3.7.1 (MN-2022), 6.EE.A.3 (CCSS-M), 6.NS.B.2 (CCSS-M)</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
@@ -1073,7 +1093,11 @@
           <t>Multiplying Multi-Digit Numbers</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.3, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.6, 6.3.7.1</t>
+        </is>
+      </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
           <t>6.EE.A.3</t>
@@ -1081,7 +1105,7 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.3 (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.6 (MN-2022), 6.3.7.1 (MN-2022), 6.EE.A.3 (CCSS-M)</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -1104,7 +1128,11 @@
           <t>Defining Greatest Common Factor</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
           <t>6.NS.B.4</t>
@@ -1112,7 +1140,7 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.B.4 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022), 6.NS.B.4 (CCSS-M)</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
@@ -1135,7 +1163,11 @@
           <t>Understanding the Distributive Property</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr"/>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.3, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.6, 6.3.7.1</t>
+        </is>
+      </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
           <t>6.EE.A.3</t>
@@ -1143,7 +1175,7 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.3 (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.6 (MN-2022), 6.3.7.1 (MN-2022), 6.EE.A.3 (CCSS-M)</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -1284,7 +1316,11 @@
           <t>Representing Portions in Multiple Ways</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr"/>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
           <t>6.NS.B.3</t>
@@ -1292,7 +1328,7 @@
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.NS.B.3 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022), 6.NS.B.3 (CCSS-M)</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
@@ -1573,7 +1609,11 @@
           <t>Writing Equivalent Expressions</t>
         </is>
       </c>
-      <c r="D37" s="8" t="inlineStr"/>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.3, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.6, 6.3.7.1</t>
+        </is>
+      </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
           <t>6.EE.A.4, 6.EE.B.6</t>
@@ -1581,7 +1621,7 @@
       </c>
       <c r="F37" s="8" t="inlineStr">
         <is>
-          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.EE.A.4 (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.6 (MN-2022), 6.3.7.1 (MN-2022), 6.EE.A.4 (CCSS-M), 6.EE.B.6 (CCSS-M)</t>
         </is>
       </c>
       <c r="G37" s="8" t="inlineStr">
@@ -1639,7 +1679,11 @@
           <t>Using Scale Factor for Enlargement</t>
         </is>
       </c>
-      <c r="D39" s="8" t="inlineStr"/>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.2, 6.3.5.3, 6.3.5.6, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.5, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
           <t>6.RP.A.1</t>
@@ -1647,7 +1691,7 @@
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.RP.A.1 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.5 (MN-2022), 6.3.6.6 (MN-2022), 6.RP.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G39" s="8" t="inlineStr">
@@ -1670,7 +1714,11 @@
           <t>Using Scale Factor for Enlargement and Reduction</t>
         </is>
       </c>
-      <c r="D40" s="8" t="inlineStr"/>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.2, 6.3.5.3, 6.3.5.6, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.5, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
           <t>6.RP.A.1</t>
@@ -1678,7 +1726,7 @@
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.RP.A.1 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.5 (MN-2022), 6.3.6.6 (MN-2022), 6.RP.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
@@ -1701,7 +1749,11 @@
           <t>Using Ratios to Compare Similar Figures</t>
         </is>
       </c>
-      <c r="D41" s="8" t="inlineStr"/>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.2, 6.3.5.3, 6.3.5.6, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.5, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
           <t>6.RP.A.1</t>
@@ -1709,7 +1761,7 @@
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.RP.A.1 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.5 (MN-2022), 6.3.6.6 (MN-2022), 6.RP.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
@@ -1732,7 +1784,11 @@
           <t>Using Ratios that Apply to Different Contexts</t>
         </is>
       </c>
-      <c r="D42" s="8" t="inlineStr"/>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.2, 6.3.5.3, 6.3.5.6, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.5, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
           <t>6.RP.A.1</t>
@@ -1740,7 +1796,7 @@
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.RP.A.1 (CCSS-M)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.5 (MN-2022), 6.3.6.6 (MN-2022), 6.RP.A.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr">
@@ -1811,11 +1867,15 @@
           <t>Representing Fraction Multiplication</t>
         </is>
       </c>
-      <c r="D45" s="8" t="inlineStr"/>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E45" s="8" t="inlineStr"/>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -1873,7 +1933,11 @@
           <t>Multiplying Mixed Numbers</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr"/>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
           <t>Review skills needed for 6.NS.1</t>
@@ -1881,7 +1945,7 @@
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), Review skills needed for 6.NS.1 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
@@ -1939,7 +2003,11 @@
           <t>Fraction Multiplication Number Sense</t>
         </is>
       </c>
-      <c r="D49" s="8" t="inlineStr"/>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
           <t>Review skills needed for 6.NS.1</t>
@@ -1947,7 +2015,7 @@
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), Review skills needed for 6.NS.1 (CCSS-M)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022), Review skills needed for 6.NS.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
@@ -1970,7 +2038,11 @@
           <t>Decompose shapes into rectangles to find area</t>
         </is>
       </c>
-      <c r="D50" s="8" t="inlineStr"/>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>6.2.3.1, 6.2.3.2, 6.2.3.3, 6.2.3.4, 6.2.3.5, 6.2.4.1, 6.2.4.2, 6.2.4.3</t>
+        </is>
+      </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
           <t>6.G.1</t>
@@ -1978,7 +2050,7 @@
       </c>
       <c r="F50" s="8" t="inlineStr">
         <is>
-          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
+          <t>6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022), 6.2.3.3 (MN-2022), 6.2.3.4 (MN-2022), 6.2.3.5 (MN-2022), 6.2.4.1 (MN-2022), 6.2.4.2 (MN-2022), 6.2.4.3 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G50" s="8" t="inlineStr">
@@ -2001,7 +2073,11 @@
           <t>Area of Parallelogram</t>
         </is>
       </c>
-      <c r="D51" s="8" t="inlineStr"/>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>6.2.3.1, 6.2.3.2, 6.2.3.3, 6.2.3.4, 6.2.3.5, 6.2.4.1, 6.2.4.2, 6.2.4.3</t>
+        </is>
+      </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
           <t>6.G.1</t>
@@ -2009,7 +2085,7 @@
       </c>
       <c r="F51" s="8" t="inlineStr">
         <is>
-          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
+          <t>6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022), 6.2.3.3 (MN-2022), 6.2.3.4 (MN-2022), 6.2.3.5 (MN-2022), 6.2.4.1 (MN-2022), 6.2.4.2 (MN-2022), 6.2.4.3 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
@@ -2032,7 +2108,11 @@
           <t>Area of Triangles</t>
         </is>
       </c>
-      <c r="D52" s="8" t="inlineStr"/>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>6.2.3.1, 6.2.3.2, 6.2.3.3, 6.2.3.4, 6.2.3.5, 6.2.4.1, 6.2.4.2, 6.2.4.3</t>
+        </is>
+      </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
           <t>6.G.1</t>
@@ -2040,7 +2120,7 @@
       </c>
       <c r="F52" s="8" t="inlineStr">
         <is>
-          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
+          <t>6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022), 6.2.3.3 (MN-2022), 6.2.3.4 (MN-2022), 6.2.3.5 (MN-2022), 6.2.4.1 (MN-2022), 6.2.4.2 (MN-2022), 6.2.4.3 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G52" s="8" t="inlineStr">
@@ -2063,7 +2143,11 @@
           <t>Area of Trapezoids</t>
         </is>
       </c>
-      <c r="D53" s="8" t="inlineStr"/>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>6.2.3.1, 6.2.3.2, 6.2.3.3, 6.2.3.4, 6.2.3.5, 6.2.4.1, 6.2.4.2, 6.2.4.3</t>
+        </is>
+      </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
           <t>6.G.1</t>
@@ -2071,7 +2155,7 @@
       </c>
       <c r="F53" s="8" t="inlineStr">
         <is>
-          <t>6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
+          <t>6.2.3.1 (MN-2022), 6.2.3.2 (MN-2022), 6.2.3.3 (MN-2022), 6.2.3.4 (MN-2022), 6.2.3.5 (MN-2022), 6.2.4.1 (MN-2022), 6.2.4.2 (MN-2022), 6.2.4.3 (MN-2022), 6.3.1.1 (MN-2007), 6.3.1.2 (MN-2007), 6.G.1 (CCSS-M)</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
@@ -2107,11 +2191,15 @@
           <t>Quotients can be expressed as addition expressions, fractions greater than 1, and mixed numbers</t>
         </is>
       </c>
-      <c r="D55" s="8" t="inlineStr"/>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.3, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.6, 6.3.7.1</t>
+        </is>
+      </c>
       <c r="E55" s="8" t="inlineStr"/>
       <c r="F55" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.6 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G55" s="8" t="inlineStr">
@@ -2134,11 +2222,15 @@
           <t>Consider meanings of numbers in a division problem as what they represent changes</t>
         </is>
       </c>
-      <c r="D56" s="8" t="inlineStr"/>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E56" s="8" t="inlineStr"/>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
@@ -2161,11 +2253,15 @@
           <t>Dividing by unit fractions is equivalent to multiplying by the denominator</t>
         </is>
       </c>
-      <c r="D57" s="8" t="inlineStr"/>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E57" s="8" t="inlineStr"/>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G57" s="8" t="inlineStr">
@@ -2250,11 +2346,15 @@
           <t>Algebra Tiles</t>
         </is>
       </c>
-      <c r="D60" s="8" t="inlineStr"/>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.3, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.6, 6.3.7.1</t>
+        </is>
+      </c>
       <c r="E60" s="8" t="inlineStr"/>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.6 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
@@ -2277,11 +2377,15 @@
           <t>Algebra Tiles</t>
         </is>
       </c>
-      <c r="D61" s="8" t="inlineStr"/>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.3, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.6, 6.3.7.1</t>
+        </is>
+      </c>
       <c r="E61" s="8" t="inlineStr"/>
       <c r="F61" s="8" t="inlineStr">
         <is>
-          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.6 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G61" s="8" t="inlineStr">
@@ -2304,11 +2408,15 @@
           <t>Combining Like Terms</t>
         </is>
       </c>
-      <c r="D62" s="8" t="inlineStr"/>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.3, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.6, 6.3.7.1</t>
+        </is>
+      </c>
       <c r="E62" s="8" t="inlineStr"/>
       <c r="F62" s="8" t="inlineStr">
         <is>
-          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.6 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr">
@@ -2331,11 +2439,15 @@
           <t>Evaluate expressions</t>
         </is>
       </c>
-      <c r="D63" s="8" t="inlineStr"/>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.3, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.6, 6.3.7.1</t>
+        </is>
+      </c>
       <c r="E63" s="8" t="inlineStr"/>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007)</t>
+          <t>6.2.1.1 (MN-2007), 6.2.2.1 (MN-2007), 6.2.2.2 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.6 (MN-2022), 6.3.7.1 (MN-2022)</t>
         </is>
       </c>
       <c r="G63" s="8" t="inlineStr">
@@ -2429,11 +2541,15 @@
           <t>Compare using tables and graphs</t>
         </is>
       </c>
-      <c r="D67" s="8" t="inlineStr"/>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.2, 6.3.5.3, 6.3.5.6, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.5, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E67" s="8" t="inlineStr"/>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.5 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G67" s="8" t="inlineStr">
@@ -2456,11 +2572,15 @@
           <t>Compare using unit rates</t>
         </is>
       </c>
-      <c r="D68" s="8" t="inlineStr"/>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.2, 6.3.5.3, 6.3.5.6, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.5, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E68" s="8" t="inlineStr"/>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007)</t>
+          <t>6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.6 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.5 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
@@ -2510,11 +2630,15 @@
           <t>Model fraction division</t>
         </is>
       </c>
-      <c r="D70" s="8" t="inlineStr"/>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E70" s="8" t="inlineStr"/>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G70" s="8" t="inlineStr">
@@ -2537,11 +2661,15 @@
           <t>Alternate Strategies for fraction division</t>
         </is>
       </c>
-      <c r="D71" s="8" t="inlineStr"/>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E71" s="8" t="inlineStr"/>
       <c r="F71" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G71" s="8" t="inlineStr">
@@ -2564,11 +2692,15 @@
           <t>Fraction Division Algorithm</t>
         </is>
       </c>
-      <c r="D72" s="8" t="inlineStr"/>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.5.4, 6.3.5.5, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E72" s="8" t="inlineStr"/>
       <c r="F72" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.3.5.11 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G72" s="8" t="inlineStr">
@@ -2591,11 +2723,15 @@
           <t>Fraction Division as Ratios</t>
         </is>
       </c>
-      <c r="D73" s="8" t="inlineStr"/>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.10, 6.3.5.11, 6.3.5.2, 6.3.5.3, 6.3.5.4, 6.3.5.5, 6.3.5.6, 6.3.5.7, 6.3.5.8, 6.3.5.9, 6.3.6.1, 6.3.6.2, 6.3.6.3, 6.3.6.4, 6.3.6.5, 6.3.6.6</t>
+        </is>
+      </c>
       <c r="E73" s="8" t="inlineStr"/>
       <c r="F73" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007)</t>
+          <t>6.1.1.1 (MN-2007), 6.1.1.2 (MN-2007), 6.1.1.3 (MN-2007), 6.1.1.4 (MN-2007), 6.1.2.1 (MN-2007), 6.1.2.2 (MN-2007), 6.1.2.3 (MN-2007), 6.3.5.10 (MN-2022), 6.3.5.11 (MN-2022), 6.3.5.2 (MN-2022), 6.3.5.3 (MN-2022), 6.3.5.4 (MN-2022), 6.3.5.5 (MN-2022), 6.3.5.6 (MN-2022), 6.3.5.7 (MN-2022), 6.3.5.8 (MN-2022), 6.3.5.9 (MN-2022), 6.3.6.1 (MN-2022), 6.3.6.2 (MN-2022), 6.3.6.3 (MN-2022), 6.3.6.4 (MN-2022), 6.3.6.5 (MN-2022), 6.3.6.6 (MN-2022)</t>
         </is>
       </c>
       <c r="G73" s="8" t="inlineStr">
@@ -3055,11 +3191,15 @@
           <t>Use percent knowledge to calculate discounts and sale prices</t>
         </is>
       </c>
-      <c r="D93" s="8" t="inlineStr"/>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>6.3.5.11, 6.3.6.2</t>
+        </is>
+      </c>
       <c r="E93" s="8" t="inlineStr"/>
       <c r="F93" s="8" t="inlineStr">
         <is>
-          <t>6.1.1.4 (MN-2007)</t>
+          <t>6.1.1.4 (MN-2007), 6.3.5.11 (MN-2022), 6.3.6.2 (MN-2022)</t>
         </is>
       </c>
       <c r="G93" s="8" t="inlineStr">

</xml_diff>